<commit_message>
add first supplementary table
</commit_message>
<xml_diff>
--- a/new_tables.xlsx
+++ b/new_tables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maxsalvatore/Documents/projects/covid/new_cancer/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8A2CFCF-2936-6044-A826-1C8C32713F3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED8E8BD2-3063-264F-B081-68FD5B39248D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="1" xr2:uid="{23B5B348-4D99-B540-995F-50D24F235ACD}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" activeTab="5" xr2:uid="{23B5B348-4D99-B540-995F-50D24F235ACD}"/>
   </bookViews>
   <sheets>
     <sheet name="table 1" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="table 3" sheetId="3" r:id="rId3"/>
     <sheet name="table 4" sheetId="5" r:id="rId4"/>
     <sheet name="table 5" sheetId="4" r:id="rId5"/>
+    <sheet name="cancer_counts" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="969" uniqueCount="719">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1181" uniqueCount="923">
   <si>
     <t>Age</t>
   </si>
@@ -2418,6 +2419,636 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">. Logistic regression odds ratios (95% CI) for COVID-19 outcomes by cancer and by cancer treatment type. </t>
+    </r>
+  </si>
+  <si>
+    <t>145</t>
+  </si>
+  <si>
+    <t>Cancer of mouth</t>
+  </si>
+  <si>
+    <t>145.1</t>
+  </si>
+  <si>
+    <t>Cancer of lip</t>
+  </si>
+  <si>
+    <t>145.2</t>
+  </si>
+  <si>
+    <t>Cancer of tongue</t>
+  </si>
+  <si>
+    <t>145.3</t>
+  </si>
+  <si>
+    <t>Cancer of major salivary glands</t>
+  </si>
+  <si>
+    <t>145.4</t>
+  </si>
+  <si>
+    <t>Cancer of the gums</t>
+  </si>
+  <si>
+    <t>145.5</t>
+  </si>
+  <si>
+    <t>Cancer of the mouth floor</t>
+  </si>
+  <si>
+    <t>149</t>
+  </si>
+  <si>
+    <t>Cancer of larynx, pharynx, nasal cavities</t>
+  </si>
+  <si>
+    <t>149.1</t>
+  </si>
+  <si>
+    <t>Cancer of oropharynx</t>
+  </si>
+  <si>
+    <t>149.2</t>
+  </si>
+  <si>
+    <t>Cancer of nasopharynx</t>
+  </si>
+  <si>
+    <t>149.3</t>
+  </si>
+  <si>
+    <t>Cancer of hypopharynx</t>
+  </si>
+  <si>
+    <t>149.4</t>
+  </si>
+  <si>
+    <t>Cancer of larynx</t>
+  </si>
+  <si>
+    <t>149.5</t>
+  </si>
+  <si>
+    <t>Hx of malignant neoplasm of oral cavity and pharynx</t>
+  </si>
+  <si>
+    <t>149.9</t>
+  </si>
+  <si>
+    <t>Cancer of of nasal cavities</t>
+  </si>
+  <si>
+    <t>150</t>
+  </si>
+  <si>
+    <t>Cancer of esophagus</t>
+  </si>
+  <si>
+    <t>151</t>
+  </si>
+  <si>
+    <t>Cancer of stomach</t>
+  </si>
+  <si>
+    <t>153</t>
+  </si>
+  <si>
+    <t>Colorectal cancer</t>
+  </si>
+  <si>
+    <t>153.2</t>
+  </si>
+  <si>
+    <t>Colon cancer</t>
+  </si>
+  <si>
+    <t>153.3</t>
+  </si>
+  <si>
+    <t>Malignant neoplasm of rectum, rectosigmoid junction, and anus</t>
+  </si>
+  <si>
+    <t>155</t>
+  </si>
+  <si>
+    <t>Cancer of liver and intrahepatic bile duct</t>
+  </si>
+  <si>
+    <t>155.1</t>
+  </si>
+  <si>
+    <t>Malignant neoplasm of liver, primary</t>
+  </si>
+  <si>
+    <t>157</t>
+  </si>
+  <si>
+    <t>Pancreatic cancer</t>
+  </si>
+  <si>
+    <t>158</t>
+  </si>
+  <si>
+    <t>Neoplasm of unspecified nature of digestive system</t>
+  </si>
+  <si>
+    <t>159</t>
+  </si>
+  <si>
+    <t>Malignant neoplasm of other and ill-defined sites within the digestive organs and peritoneum</t>
+  </si>
+  <si>
+    <t>159.2</t>
+  </si>
+  <si>
+    <t>Malignant neoplasm of small intestine, including duodenum</t>
+  </si>
+  <si>
+    <t>159.3</t>
+  </si>
+  <si>
+    <t>Malignant neoplasm of gallbladder and extrahepatic bile ducts</t>
+  </si>
+  <si>
+    <t>159.4</t>
+  </si>
+  <si>
+    <t>Malignant neoplasm of retroperitoneum and peritoneum</t>
+  </si>
+  <si>
+    <t>164</t>
+  </si>
+  <si>
+    <t>Cancer of intrathoracic organs</t>
+  </si>
+  <si>
+    <t>165</t>
+  </si>
+  <si>
+    <t>Cancer within the respiratory system</t>
+  </si>
+  <si>
+    <t>165.1</t>
+  </si>
+  <si>
+    <t>Cancer of bronchus; lung</t>
+  </si>
+  <si>
+    <t>170</t>
+  </si>
+  <si>
+    <t>Cancer of bone and connective tissue</t>
+  </si>
+  <si>
+    <t>170.1</t>
+  </si>
+  <si>
+    <t>Bone cancer</t>
+  </si>
+  <si>
+    <t>170.2</t>
+  </si>
+  <si>
+    <t>Cancer of connective tissue</t>
+  </si>
+  <si>
+    <t>172.1</t>
+  </si>
+  <si>
+    <t>Melanomas of skin, dx or hx</t>
+  </si>
+  <si>
+    <t>172.11</t>
+  </si>
+  <si>
+    <t>Melanomas of skin</t>
+  </si>
+  <si>
+    <t>174</t>
+  </si>
+  <si>
+    <t>174.1</t>
+  </si>
+  <si>
+    <t>Breast cancer [female]</t>
+  </si>
+  <si>
+    <t>174.11</t>
+  </si>
+  <si>
+    <t>Malignant neoplasm of female breast</t>
+  </si>
+  <si>
+    <t>174.2</t>
+  </si>
+  <si>
+    <t>Breast cancer [male]</t>
+  </si>
+  <si>
+    <t>174.3</t>
+  </si>
+  <si>
+    <t>Neoplasm of uncertain behavior of breast</t>
+  </si>
+  <si>
+    <t>175</t>
+  </si>
+  <si>
+    <t>Acquired absence of breast</t>
+  </si>
+  <si>
+    <t>180</t>
+  </si>
+  <si>
+    <t>Cervical cancer and dysplasia</t>
+  </si>
+  <si>
+    <t>180.1</t>
+  </si>
+  <si>
+    <t>Cervical cancer</t>
+  </si>
+  <si>
+    <t>180.3</t>
+  </si>
+  <si>
+    <t>Cervical intraepithelial neoplasia [CIN] [Cervical dysplasia]</t>
+  </si>
+  <si>
+    <t>182</t>
+  </si>
+  <si>
+    <t>Malignant neoplasm of uterus</t>
+  </si>
+  <si>
+    <t>184</t>
+  </si>
+  <si>
+    <t>Cancer of other female genital organs</t>
+  </si>
+  <si>
+    <t>184.1</t>
+  </si>
+  <si>
+    <t>Malignant neoplasm of ovary and other uterine adnexa</t>
+  </si>
+  <si>
+    <t>184.11</t>
+  </si>
+  <si>
+    <t>Malignant neoplasm of ovary</t>
+  </si>
+  <si>
+    <t>184.2</t>
+  </si>
+  <si>
+    <t>Cancer of other female genital organs (excluding uterus and ovary)</t>
+  </si>
+  <si>
+    <t>185</t>
+  </si>
+  <si>
+    <t>Cancer of prostate</t>
+  </si>
+  <si>
+    <t>187</t>
+  </si>
+  <si>
+    <t>Cancer of other male genital organs</t>
+  </si>
+  <si>
+    <t>187.1</t>
+  </si>
+  <si>
+    <t>Malignant neoplasm of unspecified male genital organ</t>
+  </si>
+  <si>
+    <t>187.2</t>
+  </si>
+  <si>
+    <t>Malignant neoplasm of testis</t>
+  </si>
+  <si>
+    <t>187.8</t>
+  </si>
+  <si>
+    <t>Neoplasm of uncertain behavior of male genital organs</t>
+  </si>
+  <si>
+    <t>189</t>
+  </si>
+  <si>
+    <t>Cancer of urinary organs (incl. kidney and bladder)</t>
+  </si>
+  <si>
+    <t>189.1</t>
+  </si>
+  <si>
+    <t>Cancer of kidney and renal pelvis</t>
+  </si>
+  <si>
+    <t>189.11</t>
+  </si>
+  <si>
+    <t>Malignant neoplasm of kidney, except pelvis</t>
+  </si>
+  <si>
+    <t>189.12</t>
+  </si>
+  <si>
+    <t>Malignant neoplasm of renal pelvis</t>
+  </si>
+  <si>
+    <t>189.2</t>
+  </si>
+  <si>
+    <t>Cancer of bladder</t>
+  </si>
+  <si>
+    <t>189.21</t>
+  </si>
+  <si>
+    <t>Malignant neoplasm of bladder</t>
+  </si>
+  <si>
+    <t>189.4</t>
+  </si>
+  <si>
+    <t>Malignant neoplasm of other urinary organs</t>
+  </si>
+  <si>
+    <t>190</t>
+  </si>
+  <si>
+    <t>Cancer of eye</t>
+  </si>
+  <si>
+    <t>191</t>
+  </si>
+  <si>
+    <t>Manlignant and unknown neoplasms of brain and nervous system</t>
+  </si>
+  <si>
+    <t>191.1</t>
+  </si>
+  <si>
+    <t>Cancer of brain and nervous system</t>
+  </si>
+  <si>
+    <t>191.11</t>
+  </si>
+  <si>
+    <t>Cancer of brain</t>
+  </si>
+  <si>
+    <t>193</t>
+  </si>
+  <si>
+    <t>Thyroid cancer</t>
+  </si>
+  <si>
+    <t>194</t>
+  </si>
+  <si>
+    <t>Cancer of other endocrine glands</t>
+  </si>
+  <si>
+    <t>195</t>
+  </si>
+  <si>
+    <t>Cancer, suspected or other</t>
+  </si>
+  <si>
+    <t>195.1</t>
+  </si>
+  <si>
+    <t>Malignant neoplasm, other</t>
+  </si>
+  <si>
+    <t>195.3</t>
+  </si>
+  <si>
+    <t>Malignant neoplasm of head, face, and neck</t>
+  </si>
+  <si>
+    <t>196</t>
+  </si>
+  <si>
+    <t>Radiotherapy</t>
+  </si>
+  <si>
+    <t>197</t>
+  </si>
+  <si>
+    <t>198</t>
+  </si>
+  <si>
+    <t>Secondary malignant neoplasm</t>
+  </si>
+  <si>
+    <t>198.1</t>
+  </si>
+  <si>
+    <t>Secondary malignancy of lymph nodes</t>
+  </si>
+  <si>
+    <t>198.2</t>
+  </si>
+  <si>
+    <t>Secondary malignancy of respiratory organs</t>
+  </si>
+  <si>
+    <t>198.3</t>
+  </si>
+  <si>
+    <t>Secondary malignant neoplasm of digestive systems</t>
+  </si>
+  <si>
+    <t>198.4</t>
+  </si>
+  <si>
+    <t>Secondary malignant neoplasm of liver</t>
+  </si>
+  <si>
+    <t>198.5</t>
+  </si>
+  <si>
+    <t>Secondary malignancy of brain/spine</t>
+  </si>
+  <si>
+    <t>198.6</t>
+  </si>
+  <si>
+    <t>Secondary malignancy of bone</t>
+  </si>
+  <si>
+    <t>198.7</t>
+  </si>
+  <si>
+    <t>Secondary malignant neoplasm of skin</t>
+  </si>
+  <si>
+    <t>199</t>
+  </si>
+  <si>
+    <t>Neoplasm of uncertain behavior</t>
+  </si>
+  <si>
+    <t>199.4</t>
+  </si>
+  <si>
+    <t>Neurofibromatosis</t>
+  </si>
+  <si>
+    <t>200</t>
+  </si>
+  <si>
+    <t>Myeloproliferative disease</t>
+  </si>
+  <si>
+    <t>200.1</t>
+  </si>
+  <si>
+    <t>Polycythemia vera</t>
+  </si>
+  <si>
+    <t>201</t>
+  </si>
+  <si>
+    <t>Hodgkin's disease</t>
+  </si>
+  <si>
+    <t>202</t>
+  </si>
+  <si>
+    <t>Cancer of other lymphoid, histiocytic tissue</t>
+  </si>
+  <si>
+    <t>202.2</t>
+  </si>
+  <si>
+    <t>Non-Hodgkins lymphoma</t>
+  </si>
+  <si>
+    <t>202.21</t>
+  </si>
+  <si>
+    <t>Nodular lymphoma</t>
+  </si>
+  <si>
+    <t>202.22</t>
+  </si>
+  <si>
+    <t>Reticulosarcoma</t>
+  </si>
+  <si>
+    <t>202.23</t>
+  </si>
+  <si>
+    <t>Lymphosarcoma</t>
+  </si>
+  <si>
+    <t>202.24</t>
+  </si>
+  <si>
+    <t>Large cell lymphoma</t>
+  </si>
+  <si>
+    <t>204</t>
+  </si>
+  <si>
+    <t>Leukemia</t>
+  </si>
+  <si>
+    <t>204.1</t>
+  </si>
+  <si>
+    <t>Lymphoid leukemia</t>
+  </si>
+  <si>
+    <t>204.11</t>
+  </si>
+  <si>
+    <t>Lymphoid leukemia, acute</t>
+  </si>
+  <si>
+    <t>204.12</t>
+  </si>
+  <si>
+    <t>Lymphoid leukemia, chronic</t>
+  </si>
+  <si>
+    <t>204.2</t>
+  </si>
+  <si>
+    <t>Myeloid leukemia</t>
+  </si>
+  <si>
+    <t>204.21</t>
+  </si>
+  <si>
+    <t>Myeloid leukemia, acute</t>
+  </si>
+  <si>
+    <t>204.22</t>
+  </si>
+  <si>
+    <t>Myeloid leukemia, chronic</t>
+  </si>
+  <si>
+    <t>204.3</t>
+  </si>
+  <si>
+    <t>Monocytic leukemia</t>
+  </si>
+  <si>
+    <t>204.4</t>
+  </si>
+  <si>
+    <t>Multiple myeloma</t>
+  </si>
+  <si>
+    <t>209</t>
+  </si>
+  <si>
+    <t>Neuroendocrine tumors</t>
+  </si>
+  <si>
+    <t>860</t>
+  </si>
+  <si>
+    <t>Bone marrow or stem cell transplant</t>
+  </si>
+  <si>
+    <t>Phecode</t>
+  </si>
+  <si>
+    <t>Phenotype</t>
+  </si>
+  <si>
+    <t>Count</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t>Table X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t>. Phecodes used to identify individuals with cancer, along with their phenotype description and the number of individuals in the tested positive cohort with the corresponding phecode.</t>
     </r>
   </si>
 </sst>
@@ -2621,7 +3252,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="94">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -2791,41 +3422,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2849,8 +3447,47 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3177,30 +3814,30 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.15">
-      <c r="B2" s="74" t="s">
+      <c r="B2" s="84" t="s">
         <v>449</v>
       </c>
-      <c r="C2" s="74"/>
-      <c r="D2" s="74"/>
-      <c r="E2" s="74"/>
-      <c r="F2" s="74"/>
-      <c r="G2" s="74"/>
-      <c r="H2" s="74"/>
-      <c r="I2" s="74"/>
+      <c r="C2" s="84"/>
+      <c r="D2" s="84"/>
+      <c r="E2" s="84"/>
+      <c r="F2" s="84"/>
+      <c r="G2" s="84"/>
+      <c r="H2" s="84"/>
+      <c r="I2" s="84"/>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.15">
       <c r="B3" s="4"/>
-      <c r="C3" s="71" t="s">
+      <c r="C3" s="81" t="s">
         <v>445</v>
       </c>
-      <c r="D3" s="71"/>
-      <c r="E3" s="71"/>
-      <c r="F3" s="72" t="s">
+      <c r="D3" s="81"/>
+      <c r="E3" s="81"/>
+      <c r="F3" s="82" t="s">
         <v>446</v>
       </c>
-      <c r="G3" s="73"/>
-      <c r="H3" s="73"/>
-      <c r="I3" s="73"/>
+      <c r="G3" s="83"/>
+      <c r="H3" s="83"/>
+      <c r="I3" s="83"/>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.15">
       <c r="B4" s="4"/>
@@ -5183,75 +5820,75 @@
       </c>
     </row>
     <row r="90" spans="2:9" x14ac:dyDescent="0.15">
-      <c r="B90" s="75" t="s">
+      <c r="B90" s="85" t="s">
         <v>450</v>
       </c>
-      <c r="C90" s="75"/>
-      <c r="D90" s="75"/>
-      <c r="E90" s="75"/>
-      <c r="F90" s="75"/>
-      <c r="G90" s="75"/>
-      <c r="H90" s="75"/>
-      <c r="I90" s="75"/>
+      <c r="C90" s="85"/>
+      <c r="D90" s="85"/>
+      <c r="E90" s="85"/>
+      <c r="F90" s="85"/>
+      <c r="G90" s="85"/>
+      <c r="H90" s="85"/>
+      <c r="I90" s="85"/>
     </row>
     <row r="91" spans="2:9" ht="13" x14ac:dyDescent="0.15">
-      <c r="B91" s="76" t="s">
+      <c r="B91" s="86" t="s">
         <v>451</v>
       </c>
-      <c r="C91" s="76"/>
-      <c r="D91" s="76"/>
-      <c r="E91" s="76"/>
-      <c r="F91" s="76"/>
-      <c r="G91" s="76"/>
-      <c r="H91" s="76"/>
-      <c r="I91" s="76"/>
+      <c r="C91" s="86"/>
+      <c r="D91" s="86"/>
+      <c r="E91" s="86"/>
+      <c r="F91" s="86"/>
+      <c r="G91" s="86"/>
+      <c r="H91" s="86"/>
+      <c r="I91" s="86"/>
     </row>
     <row r="92" spans="2:9" ht="37" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B92" s="77" t="s">
+      <c r="B92" s="80" t="s">
         <v>452</v>
       </c>
-      <c r="C92" s="77"/>
-      <c r="D92" s="77"/>
-      <c r="E92" s="77"/>
-      <c r="F92" s="77"/>
-      <c r="G92" s="77"/>
-      <c r="H92" s="77"/>
-      <c r="I92" s="77"/>
+      <c r="C92" s="80"/>
+      <c r="D92" s="80"/>
+      <c r="E92" s="80"/>
+      <c r="F92" s="80"/>
+      <c r="G92" s="80"/>
+      <c r="H92" s="80"/>
+      <c r="I92" s="80"/>
     </row>
     <row r="93" spans="2:9" ht="26" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B93" s="77" t="s">
+      <c r="B93" s="80" t="s">
         <v>453</v>
       </c>
-      <c r="C93" s="77"/>
-      <c r="D93" s="77"/>
-      <c r="E93" s="77"/>
-      <c r="F93" s="77"/>
-      <c r="G93" s="77"/>
-      <c r="H93" s="77"/>
-      <c r="I93" s="77"/>
+      <c r="C93" s="80"/>
+      <c r="D93" s="80"/>
+      <c r="E93" s="80"/>
+      <c r="F93" s="80"/>
+      <c r="G93" s="80"/>
+      <c r="H93" s="80"/>
+      <c r="I93" s="80"/>
     </row>
     <row r="94" spans="2:9" ht="25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B94" s="77" t="s">
+      <c r="B94" s="80" t="s">
         <v>454</v>
       </c>
-      <c r="C94" s="77"/>
-      <c r="D94" s="77"/>
-      <c r="E94" s="77"/>
-      <c r="F94" s="77"/>
-      <c r="G94" s="77"/>
-      <c r="H94" s="77"/>
-      <c r="I94" s="77"/>
+      <c r="C94" s="80"/>
+      <c r="D94" s="80"/>
+      <c r="E94" s="80"/>
+      <c r="F94" s="80"/>
+      <c r="G94" s="80"/>
+      <c r="H94" s="80"/>
+      <c r="I94" s="80"/>
     </row>
   </sheetData>
   <mergeCells count="8">
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="B90:I90"/>
+    <mergeCell ref="B91:I91"/>
     <mergeCell ref="B92:I92"/>
     <mergeCell ref="B93:I93"/>
     <mergeCell ref="B94:I94"/>
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="F3:I3"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="B90:I90"/>
-    <mergeCell ref="B91:I91"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5273,30 +5910,30 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:10" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="80" t="s">
+      <c r="B2" s="89" t="s">
         <v>718</v>
       </c>
-      <c r="C2" s="80"/>
-      <c r="D2" s="80"/>
-      <c r="E2" s="80"/>
-      <c r="F2" s="80"/>
-      <c r="G2" s="80"/>
-      <c r="H2" s="80"/>
-      <c r="I2" s="80"/>
-      <c r="J2" s="80"/>
+      <c r="C2" s="89"/>
+      <c r="D2" s="89"/>
+      <c r="E2" s="89"/>
+      <c r="F2" s="89"/>
+      <c r="G2" s="89"/>
+      <c r="H2" s="89"/>
+      <c r="I2" s="89"/>
+      <c r="J2" s="89"/>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="D3" s="78" t="s">
+      <c r="D3" s="87" t="s">
         <v>549</v>
       </c>
-      <c r="E3" s="79"/>
-      <c r="F3" s="79"/>
-      <c r="G3" s="79"/>
+      <c r="E3" s="88"/>
+      <c r="F3" s="88"/>
+      <c r="G3" s="88"/>
       <c r="H3" s="31"/>
-      <c r="I3" s="79" t="s">
+      <c r="I3" s="88" t="s">
         <v>552</v>
       </c>
-      <c r="J3" s="79"/>
+      <c r="J3" s="88"/>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B4" s="32" t="s">
@@ -5910,17 +6547,17 @@
       </c>
     </row>
     <row r="29" spans="2:10" ht="65" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B29" s="81" t="s">
+      <c r="B29" s="90" t="s">
         <v>553</v>
       </c>
-      <c r="C29" s="82"/>
-      <c r="D29" s="82"/>
-      <c r="E29" s="82"/>
-      <c r="F29" s="82"/>
-      <c r="G29" s="82"/>
-      <c r="H29" s="82"/>
-      <c r="I29" s="82"/>
-      <c r="J29" s="82"/>
+      <c r="C29" s="91"/>
+      <c r="D29" s="91"/>
+      <c r="E29" s="91"/>
+      <c r="F29" s="91"/>
+      <c r="G29" s="91"/>
+      <c r="H29" s="91"/>
+      <c r="I29" s="91"/>
+      <c r="J29" s="91"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -5949,30 +6586,30 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B3" s="80" t="s">
+      <c r="B3" s="89" t="s">
         <v>656</v>
       </c>
-      <c r="C3" s="80"/>
-      <c r="D3" s="80"/>
-      <c r="E3" s="80"/>
-      <c r="F3" s="80"/>
-      <c r="G3" s="80"/>
-      <c r="H3" s="80"/>
-      <c r="I3" s="80"/>
-      <c r="J3" s="80"/>
+      <c r="C3" s="89"/>
+      <c r="D3" s="89"/>
+      <c r="E3" s="89"/>
+      <c r="F3" s="89"/>
+      <c r="G3" s="89"/>
+      <c r="H3" s="89"/>
+      <c r="I3" s="89"/>
+      <c r="J3" s="89"/>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="D4" s="78" t="s">
+      <c r="D4" s="87" t="s">
         <v>549</v>
       </c>
-      <c r="E4" s="79"/>
-      <c r="F4" s="79"/>
-      <c r="G4" s="79"/>
+      <c r="E4" s="88"/>
+      <c r="F4" s="88"/>
+      <c r="G4" s="88"/>
       <c r="H4" s="31"/>
-      <c r="I4" s="79" t="s">
+      <c r="I4" s="88" t="s">
         <v>552</v>
       </c>
-      <c r="J4" s="79"/>
+      <c r="J4" s="88"/>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B5" s="32" t="s">
@@ -6734,17 +7371,17 @@
       </c>
     </row>
     <row r="36" spans="2:10" ht="66" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B36" s="81" t="s">
+      <c r="B36" s="90" t="s">
         <v>657</v>
       </c>
-      <c r="C36" s="81"/>
-      <c r="D36" s="81"/>
-      <c r="E36" s="81"/>
-      <c r="F36" s="81"/>
-      <c r="G36" s="81"/>
-      <c r="H36" s="81"/>
-      <c r="I36" s="81"/>
-      <c r="J36" s="81"/>
+      <c r="C36" s="90"/>
+      <c r="D36" s="90"/>
+      <c r="E36" s="90"/>
+      <c r="F36" s="90"/>
+      <c r="G36" s="90"/>
+      <c r="H36" s="90"/>
+      <c r="I36" s="90"/>
+      <c r="J36" s="90"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -6776,48 +7413,48 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="91" t="s">
+      <c r="B2" s="92" t="s">
         <v>716</v>
       </c>
-      <c r="C2" s="91"/>
-      <c r="D2" s="91"/>
-      <c r="E2" s="91"/>
-      <c r="F2" s="91"/>
-      <c r="G2" s="91"/>
-      <c r="H2" s="91"/>
-      <c r="I2" s="91"/>
-      <c r="J2" s="91"/>
-      <c r="K2" s="91"/>
+      <c r="C2" s="92"/>
+      <c r="D2" s="92"/>
+      <c r="E2" s="92"/>
+      <c r="F2" s="92"/>
+      <c r="G2" s="92"/>
+      <c r="H2" s="92"/>
+      <c r="I2" s="92"/>
+      <c r="J2" s="92"/>
+      <c r="K2" s="92"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B3" s="31"/>
-      <c r="C3" s="79" t="s">
+      <c r="C3" s="88" t="s">
         <v>682</v>
       </c>
-      <c r="D3" s="79"/>
-      <c r="E3" s="83"/>
-      <c r="F3" s="83"/>
-      <c r="G3" s="83"/>
-      <c r="H3" s="83"/>
+      <c r="D3" s="88"/>
+      <c r="E3" s="72"/>
+      <c r="F3" s="72"/>
+      <c r="G3" s="72"/>
+      <c r="H3" s="72"/>
     </row>
     <row r="4" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B4" s="31"/>
-      <c r="C4" s="83" t="s">
+      <c r="C4" s="72" t="s">
         <v>683</v>
       </c>
-      <c r="D4" s="83" t="s">
+      <c r="D4" s="72" t="s">
         <v>684</v>
       </c>
-      <c r="E4" s="83"/>
-      <c r="F4" s="79" t="s">
+      <c r="E4" s="72"/>
+      <c r="F4" s="88" t="s">
         <v>686</v>
       </c>
-      <c r="G4" s="79"/>
-      <c r="H4" s="79"/>
-      <c r="J4" s="79" t="s">
+      <c r="G4" s="88"/>
+      <c r="H4" s="88"/>
+      <c r="J4" s="88" t="s">
         <v>552</v>
       </c>
-      <c r="K4" s="79"/>
+      <c r="K4" s="88"/>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B5" s="32" t="s">
@@ -6875,7 +7512,7 @@
       <c r="F7" s="3">
         <v>0.14000000000000001</v>
       </c>
-      <c r="G7" s="87" t="s">
+      <c r="G7" s="76" t="s">
         <v>700</v>
       </c>
       <c r="H7" s="3">
@@ -6946,7 +7583,7 @@
       </c>
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B10" s="84" t="s">
+      <c r="B10" s="73" t="s">
         <v>679</v>
       </c>
       <c r="C10" s="2"/>
@@ -6995,7 +7632,7 @@
       <c r="D12" s="1" t="s">
         <v>689</v>
       </c>
-      <c r="F12" s="88" t="s">
+      <c r="F12" s="77" t="s">
         <v>714</v>
       </c>
       <c r="G12" s="47" t="s">
@@ -7012,7 +7649,7 @@
       </c>
     </row>
     <row r="13" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B13" s="85" t="s">
+      <c r="B13" s="74" t="s">
         <v>678</v>
       </c>
       <c r="C13" s="2" t="s">
@@ -7021,14 +7658,14 @@
       <c r="D13" s="2" t="s">
         <v>697</v>
       </c>
-      <c r="E13" s="86"/>
-      <c r="F13" s="89" t="s">
+      <c r="E13" s="75"/>
+      <c r="F13" s="78" t="s">
         <v>700</v>
       </c>
-      <c r="G13" s="89" t="s">
+      <c r="G13" s="78" t="s">
         <v>700</v>
       </c>
-      <c r="H13" s="90" t="s">
+      <c r="H13" s="79" t="s">
         <v>713</v>
       </c>
       <c r="I13" s="2"/>
@@ -7232,18 +7869,18 @@
       </c>
     </row>
     <row r="22" spans="2:11" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="81" t="s">
+      <c r="B22" s="90" t="s">
         <v>715</v>
       </c>
-      <c r="C22" s="81"/>
-      <c r="D22" s="81"/>
-      <c r="E22" s="81"/>
-      <c r="F22" s="81"/>
-      <c r="G22" s="81"/>
-      <c r="H22" s="81"/>
-      <c r="I22" s="81"/>
-      <c r="J22" s="81"/>
-      <c r="K22" s="81"/>
+      <c r="C22" s="90"/>
+      <c r="D22" s="90"/>
+      <c r="E22" s="90"/>
+      <c r="F22" s="90"/>
+      <c r="G22" s="90"/>
+      <c r="H22" s="90"/>
+      <c r="I22" s="90"/>
+      <c r="J22" s="90"/>
+      <c r="K22" s="90"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -7269,32 +7906,32 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:10" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="80" t="s">
+      <c r="B2" s="89" t="s">
         <v>717</v>
       </c>
-      <c r="C2" s="80"/>
-      <c r="D2" s="80"/>
-      <c r="E2" s="80"/>
-      <c r="F2" s="80"/>
-      <c r="G2" s="80"/>
-      <c r="H2" s="80"/>
-      <c r="I2" s="80"/>
-      <c r="J2" s="80"/>
+      <c r="C2" s="89"/>
+      <c r="D2" s="89"/>
+      <c r="E2" s="89"/>
+      <c r="F2" s="89"/>
+      <c r="G2" s="89"/>
+      <c r="H2" s="89"/>
+      <c r="I2" s="89"/>
+      <c r="J2" s="89"/>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
-      <c r="D3" s="78" t="s">
+      <c r="D3" s="87" t="s">
         <v>549</v>
       </c>
-      <c r="E3" s="79"/>
-      <c r="F3" s="79"/>
-      <c r="G3" s="79"/>
+      <c r="E3" s="88"/>
+      <c r="F3" s="88"/>
+      <c r="G3" s="88"/>
       <c r="H3" s="31"/>
-      <c r="I3" s="79" t="s">
+      <c r="I3" s="88" t="s">
         <v>552</v>
       </c>
-      <c r="J3" s="79"/>
+      <c r="J3" s="88"/>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B4" s="32" t="s">
@@ -7472,17 +8109,17 @@
       </c>
     </row>
     <row r="11" spans="2:10" ht="66" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="81" t="s">
+      <c r="B11" s="90" t="s">
         <v>553</v>
       </c>
-      <c r="C11" s="82"/>
-      <c r="D11" s="82"/>
-      <c r="E11" s="82"/>
-      <c r="F11" s="82"/>
-      <c r="G11" s="82"/>
-      <c r="H11" s="82"/>
-      <c r="I11" s="82"/>
-      <c r="J11" s="82"/>
+      <c r="C11" s="91"/>
+      <c r="D11" s="91"/>
+      <c r="E11" s="91"/>
+      <c r="F11" s="91"/>
+      <c r="G11" s="91"/>
+      <c r="H11" s="91"/>
+      <c r="I11" s="91"/>
+      <c r="J11" s="91"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -7493,4 +8130,1060 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F22A83E-07CA-E848-8AFC-AD767CC22F85}">
+  <dimension ref="B3:L38"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" style="1"/>
+    <col min="2" max="2" width="9.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="86" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.83203125" style="47" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="1.83203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="9.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="61.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.83203125" style="47" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="1.83203125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="9.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="49" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6.83203125" style="47" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="10.83203125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B3" s="93" t="s">
+        <v>922</v>
+      </c>
+      <c r="C3" s="93"/>
+      <c r="D3" s="93"/>
+      <c r="E3" s="93"/>
+      <c r="F3" s="93"/>
+      <c r="G3" s="93"/>
+      <c r="H3" s="93"/>
+      <c r="I3" s="93"/>
+      <c r="J3" s="93"/>
+      <c r="K3" s="93"/>
+      <c r="L3" s="93"/>
+    </row>
+    <row r="4" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B4" s="32" t="s">
+        <v>919</v>
+      </c>
+      <c r="C4" s="32" t="s">
+        <v>920</v>
+      </c>
+      <c r="D4" s="71" t="s">
+        <v>921</v>
+      </c>
+      <c r="E4" s="32"/>
+      <c r="F4" s="32" t="s">
+        <v>919</v>
+      </c>
+      <c r="G4" s="32" t="s">
+        <v>920</v>
+      </c>
+      <c r="H4" s="71" t="s">
+        <v>921</v>
+      </c>
+      <c r="I4" s="32"/>
+      <c r="J4" s="32" t="s">
+        <v>919</v>
+      </c>
+      <c r="K4" s="32" t="s">
+        <v>920</v>
+      </c>
+      <c r="L4" s="71" t="s">
+        <v>921</v>
+      </c>
+    </row>
+    <row r="5" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B5" s="38" t="s">
+        <v>719</v>
+      </c>
+      <c r="C5" s="38" t="s">
+        <v>720</v>
+      </c>
+      <c r="D5" s="39">
+        <v>284</v>
+      </c>
+      <c r="F5" s="38" t="s">
+        <v>787</v>
+      </c>
+      <c r="G5" s="38" t="s">
+        <v>593</v>
+      </c>
+      <c r="H5" s="39">
+        <v>1247</v>
+      </c>
+      <c r="J5" s="38" t="s">
+        <v>854</v>
+      </c>
+      <c r="K5" s="38" t="s">
+        <v>855</v>
+      </c>
+      <c r="L5" s="39">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="6" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B6" s="1" t="s">
+        <v>721</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>722</v>
+      </c>
+      <c r="D6" s="48">
+        <v>18</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>788</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>789</v>
+      </c>
+      <c r="H6" s="48">
+        <v>1177</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>856</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>857</v>
+      </c>
+      <c r="L6" s="48">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="7" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B7" s="38" t="s">
+        <v>723</v>
+      </c>
+      <c r="C7" s="38" t="s">
+        <v>724</v>
+      </c>
+      <c r="D7" s="39">
+        <v>92</v>
+      </c>
+      <c r="F7" s="38" t="s">
+        <v>790</v>
+      </c>
+      <c r="G7" s="38" t="s">
+        <v>791</v>
+      </c>
+      <c r="H7" s="39">
+        <v>1144</v>
+      </c>
+      <c r="J7" s="38" t="s">
+        <v>858</v>
+      </c>
+      <c r="K7" s="38" t="s">
+        <v>480</v>
+      </c>
+      <c r="L7" s="39">
+        <v>2105</v>
+      </c>
+    </row>
+    <row r="8" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B8" s="1" t="s">
+        <v>725</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>726</v>
+      </c>
+      <c r="D8" s="48">
+        <v>76</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>792</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>793</v>
+      </c>
+      <c r="H8" s="48">
+        <v>9</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>859</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>860</v>
+      </c>
+      <c r="L8" s="48">
+        <v>1594</v>
+      </c>
+    </row>
+    <row r="9" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B9" s="38" t="s">
+        <v>727</v>
+      </c>
+      <c r="C9" s="38" t="s">
+        <v>728</v>
+      </c>
+      <c r="D9" s="39">
+        <v>23</v>
+      </c>
+      <c r="F9" s="38" t="s">
+        <v>794</v>
+      </c>
+      <c r="G9" s="38" t="s">
+        <v>795</v>
+      </c>
+      <c r="H9" s="39">
+        <v>89</v>
+      </c>
+      <c r="J9" s="38" t="s">
+        <v>861</v>
+      </c>
+      <c r="K9" s="38" t="s">
+        <v>862</v>
+      </c>
+      <c r="L9" s="39">
+        <v>907</v>
+      </c>
+    </row>
+    <row r="10" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B10" s="1" t="s">
+        <v>729</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>730</v>
+      </c>
+      <c r="D10" s="48">
+        <v>18</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>796</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>797</v>
+      </c>
+      <c r="H10" s="48">
+        <v>328</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>863</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>864</v>
+      </c>
+      <c r="L10" s="48">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="11" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B11" s="38" t="s">
+        <v>731</v>
+      </c>
+      <c r="C11" s="38" t="s">
+        <v>732</v>
+      </c>
+      <c r="D11" s="39">
+        <v>253</v>
+      </c>
+      <c r="F11" s="38" t="s">
+        <v>798</v>
+      </c>
+      <c r="G11" s="38" t="s">
+        <v>799</v>
+      </c>
+      <c r="H11" s="39">
+        <v>1281</v>
+      </c>
+      <c r="J11" s="38" t="s">
+        <v>865</v>
+      </c>
+      <c r="K11" s="38" t="s">
+        <v>866</v>
+      </c>
+      <c r="L11" s="39">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="12" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B12" s="1" t="s">
+        <v>733</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>734</v>
+      </c>
+      <c r="D12" s="48">
+        <v>84</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>800</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>801</v>
+      </c>
+      <c r="H12" s="48">
+        <v>193</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>867</v>
+      </c>
+      <c r="K12" s="1" t="s">
+        <v>868</v>
+      </c>
+      <c r="L12" s="48">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="13" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B13" s="38" t="s">
+        <v>735</v>
+      </c>
+      <c r="C13" s="38" t="s">
+        <v>736</v>
+      </c>
+      <c r="D13" s="39">
+        <v>30</v>
+      </c>
+      <c r="F13" s="38" t="s">
+        <v>802</v>
+      </c>
+      <c r="G13" s="38" t="s">
+        <v>803</v>
+      </c>
+      <c r="H13" s="39">
+        <v>1139</v>
+      </c>
+      <c r="J13" s="38" t="s">
+        <v>869</v>
+      </c>
+      <c r="K13" s="38" t="s">
+        <v>870</v>
+      </c>
+      <c r="L13" s="39">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="14" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B14" s="1" t="s">
+        <v>737</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>738</v>
+      </c>
+      <c r="D14" s="48">
+        <v>19</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>804</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>805</v>
+      </c>
+      <c r="H14" s="48">
+        <v>262</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>871</v>
+      </c>
+      <c r="K14" s="1" t="s">
+        <v>872</v>
+      </c>
+      <c r="L14" s="48">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="15" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B15" s="38" t="s">
+        <v>739</v>
+      </c>
+      <c r="C15" s="38" t="s">
+        <v>740</v>
+      </c>
+      <c r="D15" s="39">
+        <v>78</v>
+      </c>
+      <c r="F15" s="38" t="s">
+        <v>806</v>
+      </c>
+      <c r="G15" s="38" t="s">
+        <v>807</v>
+      </c>
+      <c r="H15" s="39">
+        <v>466</v>
+      </c>
+      <c r="J15" s="38" t="s">
+        <v>873</v>
+      </c>
+      <c r="K15" s="38" t="s">
+        <v>874</v>
+      </c>
+      <c r="L15" s="39">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="16" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B16" s="1" t="s">
+        <v>741</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>742</v>
+      </c>
+      <c r="D16" s="48">
+        <v>69</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>808</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>809</v>
+      </c>
+      <c r="H16" s="48">
+        <v>207</v>
+      </c>
+      <c r="J16" s="1" t="s">
+        <v>875</v>
+      </c>
+      <c r="K16" s="1" t="s">
+        <v>876</v>
+      </c>
+      <c r="L16" s="48">
+        <v>2595</v>
+      </c>
+    </row>
+    <row r="17" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B17" s="38" t="s">
+        <v>743</v>
+      </c>
+      <c r="C17" s="38" t="s">
+        <v>744</v>
+      </c>
+      <c r="D17" s="39">
+        <v>38</v>
+      </c>
+      <c r="F17" s="38" t="s">
+        <v>810</v>
+      </c>
+      <c r="G17" s="38" t="s">
+        <v>811</v>
+      </c>
+      <c r="H17" s="39">
+        <v>159</v>
+      </c>
+      <c r="J17" s="38" t="s">
+        <v>877</v>
+      </c>
+      <c r="K17" s="38" t="s">
+        <v>878</v>
+      </c>
+      <c r="L17" s="39">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="18" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B18" s="1" t="s">
+        <v>745</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>746</v>
+      </c>
+      <c r="D18" s="48">
+        <v>112</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>812</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>813</v>
+      </c>
+      <c r="H18" s="48">
+        <v>229</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>879</v>
+      </c>
+      <c r="K18" s="1" t="s">
+        <v>880</v>
+      </c>
+      <c r="L18" s="48">
+        <v>1215</v>
+      </c>
+    </row>
+    <row r="19" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B19" s="38" t="s">
+        <v>747</v>
+      </c>
+      <c r="C19" s="38" t="s">
+        <v>748</v>
+      </c>
+      <c r="D19" s="39">
+        <v>154</v>
+      </c>
+      <c r="F19" s="38" t="s">
+        <v>814</v>
+      </c>
+      <c r="G19" s="38" t="s">
+        <v>815</v>
+      </c>
+      <c r="H19" s="39">
+        <v>1058</v>
+      </c>
+      <c r="J19" s="38" t="s">
+        <v>881</v>
+      </c>
+      <c r="K19" s="38" t="s">
+        <v>882</v>
+      </c>
+      <c r="L19" s="39">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="20" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B20" s="1" t="s">
+        <v>749</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>750</v>
+      </c>
+      <c r="D20" s="48">
+        <v>637</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>816</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>817</v>
+      </c>
+      <c r="H20" s="48">
+        <v>158</v>
+      </c>
+      <c r="J20" s="1" t="s">
+        <v>883</v>
+      </c>
+      <c r="K20" s="1" t="s">
+        <v>884</v>
+      </c>
+      <c r="L20" s="48">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="21" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B21" s="38" t="s">
+        <v>751</v>
+      </c>
+      <c r="C21" s="38" t="s">
+        <v>752</v>
+      </c>
+      <c r="D21" s="39">
+        <v>499</v>
+      </c>
+      <c r="F21" s="38" t="s">
+        <v>818</v>
+      </c>
+      <c r="G21" s="38" t="s">
+        <v>819</v>
+      </c>
+      <c r="H21" s="39">
+        <v>29</v>
+      </c>
+      <c r="J21" s="38" t="s">
+        <v>885</v>
+      </c>
+      <c r="K21" s="38" t="s">
+        <v>886</v>
+      </c>
+      <c r="L21" s="39">
+        <v>984</v>
+      </c>
+    </row>
+    <row r="22" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B22" s="1" t="s">
+        <v>753</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>754</v>
+      </c>
+      <c r="D22" s="48">
+        <v>335</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>820</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>821</v>
+      </c>
+      <c r="H22" s="48">
+        <v>101</v>
+      </c>
+      <c r="J22" s="1" t="s">
+        <v>887</v>
+      </c>
+      <c r="K22" s="1" t="s">
+        <v>888</v>
+      </c>
+      <c r="L22" s="48">
+        <v>864</v>
+      </c>
+    </row>
+    <row r="23" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B23" s="38" t="s">
+        <v>755</v>
+      </c>
+      <c r="C23" s="38" t="s">
+        <v>756</v>
+      </c>
+      <c r="D23" s="39">
+        <v>219</v>
+      </c>
+      <c r="F23" s="38" t="s">
+        <v>822</v>
+      </c>
+      <c r="G23" s="38" t="s">
+        <v>823</v>
+      </c>
+      <c r="H23" s="39">
+        <v>40</v>
+      </c>
+      <c r="J23" s="38" t="s">
+        <v>889</v>
+      </c>
+      <c r="K23" s="38" t="s">
+        <v>890</v>
+      </c>
+      <c r="L23" s="39">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="24" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B24" s="1" t="s">
+        <v>757</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>758</v>
+      </c>
+      <c r="D24" s="48">
+        <v>172</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>824</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>825</v>
+      </c>
+      <c r="H24" s="48">
+        <v>852</v>
+      </c>
+      <c r="J24" s="1" t="s">
+        <v>891</v>
+      </c>
+      <c r="K24" s="1" t="s">
+        <v>892</v>
+      </c>
+      <c r="L24" s="48">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="25" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B25" s="38" t="s">
+        <v>759</v>
+      </c>
+      <c r="C25" s="38" t="s">
+        <v>760</v>
+      </c>
+      <c r="D25" s="39">
+        <v>133</v>
+      </c>
+      <c r="F25" s="38" t="s">
+        <v>826</v>
+      </c>
+      <c r="G25" s="38" t="s">
+        <v>827</v>
+      </c>
+      <c r="H25" s="39">
+        <v>449</v>
+      </c>
+      <c r="J25" s="38" t="s">
+        <v>893</v>
+      </c>
+      <c r="K25" s="38" t="s">
+        <v>894</v>
+      </c>
+      <c r="L25" s="39">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="26" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B26" s="1" t="s">
+        <v>761</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>762</v>
+      </c>
+      <c r="D26" s="48">
+        <v>645</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>828</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>829</v>
+      </c>
+      <c r="H26" s="48">
+        <v>383</v>
+      </c>
+      <c r="J26" s="1" t="s">
+        <v>895</v>
+      </c>
+      <c r="K26" s="1" t="s">
+        <v>896</v>
+      </c>
+      <c r="L26" s="48">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="27" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B27" s="38" t="s">
+        <v>763</v>
+      </c>
+      <c r="C27" s="38" t="s">
+        <v>764</v>
+      </c>
+      <c r="D27" s="39">
+        <v>669</v>
+      </c>
+      <c r="F27" s="38" t="s">
+        <v>830</v>
+      </c>
+      <c r="G27" s="38" t="s">
+        <v>831</v>
+      </c>
+      <c r="H27" s="39">
+        <v>50</v>
+      </c>
+      <c r="J27" s="38" t="s">
+        <v>897</v>
+      </c>
+      <c r="K27" s="38" t="s">
+        <v>898</v>
+      </c>
+      <c r="L27" s="39">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="28" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B28" s="1" t="s">
+        <v>765</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>766</v>
+      </c>
+      <c r="D28" s="48">
+        <v>57</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>832</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>833</v>
+      </c>
+      <c r="H28" s="48">
+        <v>444</v>
+      </c>
+      <c r="J28" s="1" t="s">
+        <v>899</v>
+      </c>
+      <c r="K28" s="1" t="s">
+        <v>900</v>
+      </c>
+      <c r="L28" s="48">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="29" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B29" s="38" t="s">
+        <v>767</v>
+      </c>
+      <c r="C29" s="38" t="s">
+        <v>768</v>
+      </c>
+      <c r="D29" s="39">
+        <v>37</v>
+      </c>
+      <c r="F29" s="38" t="s">
+        <v>834</v>
+      </c>
+      <c r="G29" s="38" t="s">
+        <v>835</v>
+      </c>
+      <c r="H29" s="39">
+        <v>397</v>
+      </c>
+      <c r="J29" s="38" t="s">
+        <v>901</v>
+      </c>
+      <c r="K29" s="38" t="s">
+        <v>902</v>
+      </c>
+      <c r="L29" s="39">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="30" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B30" s="1" t="s">
+        <v>769</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>770</v>
+      </c>
+      <c r="D30" s="48">
+        <v>81</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>836</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>837</v>
+      </c>
+      <c r="H30" s="48">
+        <v>111</v>
+      </c>
+      <c r="J30" s="1" t="s">
+        <v>903</v>
+      </c>
+      <c r="K30" s="1" t="s">
+        <v>904</v>
+      </c>
+      <c r="L30" s="48">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="31" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B31" s="38" t="s">
+        <v>771</v>
+      </c>
+      <c r="C31" s="38" t="s">
+        <v>772</v>
+      </c>
+      <c r="D31" s="39">
+        <v>61</v>
+      </c>
+      <c r="F31" s="38" t="s">
+        <v>838</v>
+      </c>
+      <c r="G31" s="38" t="s">
+        <v>839</v>
+      </c>
+      <c r="H31" s="39">
+        <v>81</v>
+      </c>
+      <c r="J31" s="38" t="s">
+        <v>905</v>
+      </c>
+      <c r="K31" s="38" t="s">
+        <v>906</v>
+      </c>
+      <c r="L31" s="39">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="32" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B32" s="1" t="s">
+        <v>773</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>774</v>
+      </c>
+      <c r="D32" s="48">
+        <v>459</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>840</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>841</v>
+      </c>
+      <c r="H32" s="48">
+        <v>370</v>
+      </c>
+      <c r="J32" s="1" t="s">
+        <v>907</v>
+      </c>
+      <c r="K32" s="1" t="s">
+        <v>908</v>
+      </c>
+      <c r="L32" s="48">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="33" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B33" s="38" t="s">
+        <v>775</v>
+      </c>
+      <c r="C33" s="38" t="s">
+        <v>776</v>
+      </c>
+      <c r="D33" s="39">
+        <v>397</v>
+      </c>
+      <c r="F33" s="38" t="s">
+        <v>842</v>
+      </c>
+      <c r="G33" s="38" t="s">
+        <v>843</v>
+      </c>
+      <c r="H33" s="39">
+        <v>229</v>
+      </c>
+      <c r="J33" s="38" t="s">
+        <v>909</v>
+      </c>
+      <c r="K33" s="38" t="s">
+        <v>910</v>
+      </c>
+      <c r="L33" s="39">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="34" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B34" s="1" t="s">
+        <v>777</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>778</v>
+      </c>
+      <c r="D34" s="48">
+        <v>525</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>844</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>845</v>
+      </c>
+      <c r="H34" s="48">
+        <v>199</v>
+      </c>
+      <c r="J34" s="1" t="s">
+        <v>911</v>
+      </c>
+      <c r="K34" s="1" t="s">
+        <v>912</v>
+      </c>
+      <c r="L34" s="48">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="35" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B35" s="38" t="s">
+        <v>779</v>
+      </c>
+      <c r="C35" s="38" t="s">
+        <v>780</v>
+      </c>
+      <c r="D35" s="39">
+        <v>203</v>
+      </c>
+      <c r="F35" s="38" t="s">
+        <v>846</v>
+      </c>
+      <c r="G35" s="38" t="s">
+        <v>847</v>
+      </c>
+      <c r="H35" s="39">
+        <v>371</v>
+      </c>
+      <c r="J35" s="38" t="s">
+        <v>913</v>
+      </c>
+      <c r="K35" s="38" t="s">
+        <v>914</v>
+      </c>
+      <c r="L35" s="39">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="36" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B36" s="1" t="s">
+        <v>781</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>782</v>
+      </c>
+      <c r="D36" s="48">
+        <v>392</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>848</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>849</v>
+      </c>
+      <c r="H36" s="48">
+        <v>274</v>
+      </c>
+      <c r="J36" s="1" t="s">
+        <v>915</v>
+      </c>
+      <c r="K36" s="1" t="s">
+        <v>916</v>
+      </c>
+      <c r="L36" s="48">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="37" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B37" s="38" t="s">
+        <v>783</v>
+      </c>
+      <c r="C37" s="38" t="s">
+        <v>784</v>
+      </c>
+      <c r="D37" s="39">
+        <v>1958</v>
+      </c>
+      <c r="F37" s="38" t="s">
+        <v>850</v>
+      </c>
+      <c r="G37" s="38" t="s">
+        <v>851</v>
+      </c>
+      <c r="H37" s="39">
+        <v>7030</v>
+      </c>
+      <c r="J37" s="38" t="s">
+        <v>917</v>
+      </c>
+      <c r="K37" s="38" t="s">
+        <v>918</v>
+      </c>
+      <c r="L37" s="39">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="38" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B38" s="2" t="s">
+        <v>785</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>786</v>
+      </c>
+      <c r="D38" s="45">
+        <v>834</v>
+      </c>
+      <c r="E38" s="2"/>
+      <c r="F38" s="2" t="s">
+        <v>852</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>853</v>
+      </c>
+      <c r="H38" s="45">
+        <v>6897</v>
+      </c>
+      <c r="I38" s="2"/>
+      <c r="J38" s="2"/>
+      <c r="K38" s="2"/>
+      <c r="L38" s="44"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B3:L3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>